<commit_message>
Update rainfall map analysis legends, categories, admin shortcut (Ctrl+H), and district click interaction
</commit_message>
<xml_diff>
--- a/sample-files/sample_realised_june_2025.xlsx
+++ b/sample-files/sample_realised_june_2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/divesh/Desktop/sample-files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/divesh/Desktop/imd copy/sample-files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B3C137-69F0-FB4B-87BE-21D3EC24320E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44B438CB-7079-484F-AC52-6F4E71CF9E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>